<commit_message>
Precios: Restructuracion producto_id a presentacion_id
</commit_message>
<xml_diff>
--- a/public/plantillas/plantilla_precios.xlsx
+++ b/public/plantillas/plantilla_precios.xlsx
@@ -1,20 +1,20 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios" sheetId="1" state="visible" r:id="rId1"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel</Application>
+  <AppVersion>3.0</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
+  <dc:creator xmlns:dc="http://purl.org/dc/elements/1.1/">openpyxl</dc:creator>
+  <dcterms:created xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2025-12-11T03:33:48Z</dcterms:created>
+  <dcterms:modified xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2025-12-11T03:33:48Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="1">
@@ -124,7 +124,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -407,13 +407,28 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios" sheetId="1" state="visible" r:id="rId1"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,25 +439,30 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>presentacion</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>valor_medida</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>unidad_medida</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>fecha_vigencia_inicio</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>fecha_vigencia_final</t>
         </is>
@@ -454,23 +474,28 @@
           <t>Coca-Cola</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Lata 600 ml</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>600</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>ml</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>15.5</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>2025-01-05</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -478,23 +503,28 @@
           <t>Spaghetti</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paquete 500 g</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>500</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>g</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>19</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>2025-01-10</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>2025-12-31</t>
         </is>
@@ -506,23 +536,28 @@
           <t>Azúcar Morena</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paquete 1 kg</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>28</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>2025-01-02</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>